<commit_message>
some features are added
</commit_message>
<xml_diff>
--- a/dataset_chatbot_nara.xlsx
+++ b/dataset_chatbot_nara.xlsx
@@ -10,6 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Google Classroom" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quizizz" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Moodle" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bantuan" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -41,7 +42,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -69,6 +70,12 @@
         <bgColor rgb="004472C4"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C0504D"/>
+        <bgColor rgb="00C0504D"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -82,7 +89,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -98,6 +105,9 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2521,4 +2531,465 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C26"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="32" customWidth="1" min="1" max="1"/>
+    <col width="45" customWidth="1" min="2" max="2"/>
+    <col width="85" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="6" t="inlineStr">
+        <is>
+          <t>tag</t>
+        </is>
+      </c>
+      <c r="B1" s="6" t="inlineStr">
+        <is>
+          <t>pattern</t>
+        </is>
+      </c>
+      <c r="C1" s="6" t="inlineStr">
+        <is>
+          <t>response</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="5" t="inlineStr">
+        <is>
+          <t>bantuan_gc_login</t>
+        </is>
+      </c>
+      <c r="B2" s="5" t="inlineStr">
+        <is>
+          <t>tidak bisa login google classroom</t>
+        </is>
+      </c>
+      <c r="C2" s="5" t="inlineStr">
+        <is>
+          <t>Pastikan Anda menggunakan akun yang benar. Google Classroom mendukung: (1) Akun sekolah (Google Workspace for Education, contoh: nama@sekolah.edu), (2) Akun Google pribadi. Pastikan koneksi internet aktif. Jika masih gagal, hubungi admin sekolah karena mungkin Classroom belum diaktifkan untuk akun Anda.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>bantuan_gc_login</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>gagal masuk google classroom</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>Coba langkah berikut: (1) Pastikan akun email yang digunakan sudah terdaftar di Classroom, (2) Periksa koneksi internet, (3) Coba buka classroom.google.com di browser lain, (4) Jika menggunakan akun sekolah dan tetap gagal, minta guru menghubungi admin IT sekolah.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>bantuan_gc_lupa_password</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>lupa password google classroom</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>Jika menggunakan akun Google Workspace sekolah: minta guru/admin sekolah untuk mereset password Anda. Jika menggunakan akun Google pribadi: buka accounts.google.com, klik Lupa password, lalu ikuti langkah pemulihan melalui email atau nomor HP yang terdaftar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>bantuan_gc_kode_kelas</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>kode kelas google classroom tidak berfungsi</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>Pastikan: (1) Login dengan akun yang benar, (2) Kode terdiri dari 6-8 karakter huruf dan angka tanpa spasi atau karakter khusus, (3) Perhatikan huruf kapital pada kode. Jika masih bermasalah, minta guru membagikan ulang kode kelas atau mengirim undangan lewat email.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>bantuan_gc_kode_kelas</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>lupa kode kelas google classroom</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>Kode kelas hanya diperlukan sekali saat pertama bergabung. Jika belum bergabung dan lupa kodenya, hubungi langsung guru untuk meminta kode baru atau minta guru mengirim undangan melalui email.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>bantuan_gc_upload</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>tidak bisa upload tugas google classroom</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>Coba langkah berikut: (1) Salin isi tugas ke dokumen baru, (2) Di tugas Classroom, hapus lampiran lama lalu buat salinan baru, (3) Tempelkan isi tugas ke file baru, (4) Klik Serahkan. Alternatif: lampirkan file melalui Forum lalu tautkan linknya ke tugas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>bantuan_gc_upload</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>tombol serahkan tidak berfungsi google classroom</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>Jika muncul pesan error saat klik Serahkan: (1) Coba refresh halaman, (2) Gunakan browser lain (Chrome disarankan), (3) Pastikan file tidak melebihi batas ukuran, (4) Coba upload ulang file, (5) Jika masih gagal, beritahu guru Anda.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>bantuan_gc_komentar</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>tidak bisa komentar di google classroom</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>Kemungkinan guru telah menonaktifkan fitur komentar untuk kelas tersebut. Hubungi guru Anda untuk informasi lebih lanjut atau gunakan cara lain untuk berkomunikasi dengan guru.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>bantuan_gc_email</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>tidak bisa kirim email di google classroom</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>Kemungkinan admin sekolah menonaktifkan Gmail untuk siswa. Minta guru menghubungi admin IT sekolah. Untuk akun Google pribadi, cek pengaturan Gmail atau buka Bantuan Gmail di support.google.com/mail.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>bantuan_gc_undangan</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>undangan kelas google classroom terhapus</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>Jika undangan kelas terhapus sebelum Anda bergabung, minta guru untuk mengirim ulang undangan kelas ke email Anda. Anda hanya perlu menggunakan undangan sekali untuk bergabung ke kelas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>bantuan_qz_login</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>tidak bisa login quizizz</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>Coba langkah berikut: (1) Pastikan email dan password sudah benar, (2) Coba klik Lupa Password di halaman login, (3) Periksa folder spam email untuk link verifikasi, (4) Coba login menggunakan akun Google jika sebelumnya mendaftar dengan Google, (5) Coba buka quizizz.com di browser lain atau mode incognito.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>bantuan_qz_login</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>akun quizizz tidak bisa masuk</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>Jika menggunakan akun belajar.id: pastikan akun belajar.id sudah aktif dan email sudah diverifikasi. Coba login lewat tombol 'Masuk dengan Google' menggunakan email belajar.id. Jika masih bermasalah, hubungi operator sekolah untuk memastikan akun belajar.id aktif.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>bantuan_qz_lupa_password</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>lupa password quizizz</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>Di halaman login Quizizz, klik Forgot Password, masukkan email yang terdaftar, lalu cek kotak masuk email Anda untuk link reset password. Periksa juga folder spam. Jika tidak menerima email, pastikan email yang dimasukkan sudah benar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>bantuan_qz_kuis</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>kuis quizizz tidak muncul</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>Kemungkinan penyebab: (1) Kuis belum dimulai oleh guru, (2) Kode kuis salah atau sudah kadaluarsa, (3) Coba refresh halaman, (4) Pastikan bergabung dengan kode yang diberikan guru. Hubungi guru untuk memastikan kuis sudah diaktifkan.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>bantuan_qz_kuis</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>siswa tidak bisa bergabung kuis quizizz</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>Pastikan: (1) Siswa menggunakan kode yang benar dari guru, (2) Guru sudah memulai sesi kuis, (3) Koneksi internet siswa stabil, (4) Coba buka quizizz.com langsung di browser tanpa aplikasi, (5) Coba gunakan browser Chrome untuk hasil terbaik.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>bantuan_qz_hasil</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>hasil kuis quizizz tidak tersimpan</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>Pastikan siswa menyelesaikan kuis hingga halaman hasil muncul dan tidak menutup browser di tengah kuis. Jika koneksi internet terputus saat mengerjakan, jawaban mungkin tidak tersimpan. Hubungi guru untuk meminta siswa mengulang kuis jika diperlukan.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>bantuan_moodle_login</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>tidak bisa login moodle</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>Coba langkah berikut: (1) Pastikan username dan password sudah benar, (2) Klik Lupa kata sandi di halaman login untuk reset password via email, (3) Pastikan akun sudah diaktifkan oleh admin, (4) Coba bersihkan cache browser atau gunakan browser lain, (5) Hubungi administrator Moodle sekolah jika masih gagal.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>bantuan_moodle_login</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>user tidak bisa login moodle padahal password benar</t>
+        </is>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>Masalah ini sering terjadi karena izin folder session Moodle. Solusi untuk admin: cek permission folder moodledata/sessions dan pastikan sudah diatur dengan benar. Untuk pengguna biasa: coba bersihkan cache dan cookies browser, lalu login ulang.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>bantuan_moodle_login</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>harus berkali kali login moodle baru bisa masuk</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>Masalah ini biasanya terkait session Moodle. Coba: (1) Bersihkan cache dan cookies browser, (2) Gunakan browser lain, (3) Pastikan cookies browser tidak diblokir. Untuk admin: periksa pengaturan session di Site administration &gt; Server &gt; Session handling.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>bantuan_moodle_lupa_password</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>lupa password moodle</t>
+        </is>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>Di halaman login Moodle, klik Lupa kata sandi (Forgotten your username or password?). Pilih reset via username atau email, lalu cek kotak masuk email Anda. Jika tidak menerima email, hubungi administrator Moodle sekolah untuk reset password secara manual.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>bantuan_moodle_upload</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>tidak bisa upload materi moodle</t>
+        </is>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>Pastikan: (1) Mode edit sudah diaktifkan (klik ikon Gear &gt; Turn Editing On), (2) Ukuran file tidak melebihi batas upload yang ditetapkan admin, (3) Format file didukung oleh Moodle, (4) Koneksi internet stabil saat upload. Jika masih gagal, hubungi admin untuk mengecek batas ukuran file di pengaturan Moodle.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>bantuan_moodle_upload</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="inlineStr">
+        <is>
+          <t>file tidak bisa diupload ke moodle</t>
+        </is>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>Beberapa penyebab umum: (1) Ukuran file terlalu besar (coba kompres file terlebih dahulu), (2) Format file tidak didukung, (3) Mode edit belum aktif. Minta admin untuk memeriksa pengaturan max upload size di Site administration &gt; Security &gt; Site security settings.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>bantuan_moodle_siswa_login</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="inlineStr">
+        <is>
+          <t>siswa tidak bisa login moodle</t>
+        </is>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>Pastikan: (1) Akun siswa sudah dibuat oleh admin, (2) Username dan password sudah diberikan dengan benar ke siswa, (3) Akun siswa belum dinonaktifkan. Admin dapat mengecek di Site administration &gt; Users &gt; Accounts &gt; Browse list of users untuk memverifikasi status akun siswa.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>bantuan_moodle_menu</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="inlineStr">
+        <is>
+          <t>tidak paham menu moodle</t>
+        </is>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>Menu utama Moodle terdiri dari: (1) Dashboard - halaman utama setelah login, (2) My Courses - daftar kursus yang diikuti, (3) Site administration - pengaturan sistem (khusus admin), (4) Participants - daftar peserta di kursus. Jika bingung dengan menu tertentu, klik ikon tanda tanya (?) yang tersedia di setiap halaman Moodle.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>bantuan_moodle_edit</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="inlineStr">
+        <is>
+          <t>tidak bisa edit kursus moodle</t>
+        </is>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>Pastikan mode edit sudah aktif: klik ikon Gear (roda gigi) di sebelah kanan nama kursus, lalu pilih Turn Editing On. Jika opsi ini tidak muncul, kemungkinan Anda tidak memiliki hak akses Teacher. Hubungi admin untuk memastikan peran Anda di kursus tersebut sudah diatur sebagai Teacher.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>